<commit_message>
feat: add dashboard interview management and candidate portal integration pages
</commit_message>
<xml_diff>
--- a/server/data/reports/Selected_Candidates_2026-10-12.xlsx
+++ b/server/data/reports/Selected_Candidates_2026-10-12.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="53">
   <si>
     <t>AvaHire AI - Daily Selected Candidates Report (12-Oct-2026)</t>
   </si>
   <si>
-    <t>Selection Date: 12-Oct-2026  |  Total Selected: 12 Selected Candidates  |  Generated: 12/10/2026, 14:28:24</t>
+    <t>Selection Date: 12-Oct-2026  |  Total Selected: 12 Selected Candidates  |  Generated: 12/10/2026, 19:46:51</t>
   </si>
   <si>
     <t>Sr. No.</t>
@@ -58,94 +58,85 @@
     <t>Foreign Candidate</t>
   </si>
   <si>
+    <t>foreign.1791794413159@example.com</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Product Manager</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>12 Oct 2026, 14:10</t>
+  </si>
+  <si>
+    <t>12-Oct-2026</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Selected</t>
+  </si>
+  <si>
+    <t>Download Transcript (.docx)</t>
+  </si>
+  <si>
+    <t>Download Recording (Audio)</t>
+  </si>
+  <si>
     <t>foreign.1791794342458@example.com</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Product Manager</t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
     <t>12 Oct 2026, 14:09</t>
   </si>
   <si>
-    <t>12-Oct-2026</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Selected</t>
-  </si>
-  <si>
-    <t>Download Transcript (.docx)</t>
-  </si>
-  <si>
-    <t>Download Recording (Audio)</t>
-  </si>
-  <si>
-    <t>Divya Nambiar</t>
-  </si>
-  <si>
-    <t>divya.nambiar.1791794342458@example.com</t>
-  </si>
-  <si>
-    <t>Cloud Security Specialist</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>Aakash Patel</t>
-  </si>
-  <si>
-    <t>aakash.patel.1791794342458@example.com</t>
-  </si>
-  <si>
-    <t>Senior Frontend Engineer</t>
+    <t>Aarav Sharma</t>
+  </si>
+  <si>
+    <t>aarav.sharma@example.com</t>
+  </si>
+  <si>
+    <t>+91 99887 76655</t>
+  </si>
+  <si>
+    <t>AI Research Scientist</t>
+  </si>
+  <si>
+    <t>AI/ML</t>
+  </si>
+  <si>
+    <t>User 2 Selected Candidate</t>
+  </si>
+  <si>
+    <t>u2.sel.1791791288048@test.com</t>
+  </si>
+  <si>
+    <t>DevOps Engineer</t>
+  </si>
+  <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>12 Oct 2026, 13:18</t>
+  </si>
+  <si>
+    <t>Snehal Harde</t>
+  </si>
+  <si>
+    <t>snehal.harde2935@gmail.com</t>
+  </si>
+  <si>
+    <t>+91 98765 43210</t>
+  </si>
+  <si>
+    <t>devops</t>
   </si>
   <si>
     <t>Engineering</t>
-  </si>
-  <si>
-    <t>User 2 Selected Candidate</t>
-  </si>
-  <si>
-    <t>u2.sel.1791791288048@test.com</t>
-  </si>
-  <si>
-    <t>DevOps Engineer</t>
-  </si>
-  <si>
-    <t>Infrastructure</t>
-  </si>
-  <si>
-    <t>12 Oct 2026, 13:18</t>
-  </si>
-  <si>
-    <t>User 1 Selected Candidate</t>
-  </si>
-  <si>
-    <t>u1.sel.1791791288048@test.com</t>
-  </si>
-  <si>
-    <t>Full Stack Engineer</t>
-  </si>
-  <si>
-    <t>Snehal Harde</t>
-  </si>
-  <si>
-    <t>snehal.harde2935@gmail.com</t>
-  </si>
-  <si>
-    <t>+91 98765 43210</t>
-  </si>
-  <si>
-    <t>devops</t>
   </si>
   <si>
     <t>10 Oct 2026, 11:11</t>
@@ -820,22 +811,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>20</v>
@@ -858,22 +849,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>32</v>
-      </c>
       <c r="G7" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>20</v>
@@ -896,22 +887,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>34</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="G8" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>20</v>
@@ -934,22 +925,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>20</v>
@@ -972,22 +963,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="G10" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>45</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>20</v>
@@ -1010,22 +1001,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>20</v>
@@ -1048,22 +1039,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="10" t="s">
+      <c r="G12" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>20</v>
@@ -1086,22 +1077,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>32</v>
-      </c>
       <c r="G13" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>20</v>
@@ -1124,22 +1115,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>20</v>
@@ -1162,7 +1153,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>16</v>
@@ -1171,13 +1162,13 @@
         <v>16</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>20</v>
@@ -1200,22 +1191,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="G16" s="10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>20</v>
@@ -1241,14 +1232,14 @@
   <hyperlinks>
     <hyperlink ref="K5" r:id="rId1" tooltip="Download interview transcript docx for Foreign Candidate"/>
     <hyperlink ref="L5" r:id="rId2" tooltip="Download interview audio recording for Foreign Candidate"/>
-    <hyperlink ref="K6" r:id="rId3" tooltip="Download interview transcript docx for Divya Nambiar"/>
-    <hyperlink ref="L6" r:id="rId4" tooltip="Download interview audio recording for Divya Nambiar"/>
-    <hyperlink ref="K7" r:id="rId5" tooltip="Download interview transcript docx for Aakash Patel"/>
-    <hyperlink ref="L7" r:id="rId6" tooltip="Download interview audio recording for Aakash Patel"/>
+    <hyperlink ref="K6" r:id="rId3" tooltip="Download interview transcript docx for Foreign Candidate"/>
+    <hyperlink ref="L6" r:id="rId4" tooltip="Download interview audio recording for Foreign Candidate"/>
+    <hyperlink ref="K7" r:id="rId5" tooltip="Download interview transcript docx for Aarav Sharma"/>
+    <hyperlink ref="L7" r:id="rId6" tooltip="Download interview audio recording for Aarav Sharma"/>
     <hyperlink ref="K8" r:id="rId7" tooltip="Download interview transcript docx for User 2 Selected Candidate"/>
     <hyperlink ref="L8" r:id="rId8" tooltip="Download interview audio recording for User 2 Selected Candidate"/>
-    <hyperlink ref="K9" r:id="rId9" tooltip="Download interview transcript docx for User 1 Selected Candidate"/>
-    <hyperlink ref="L9" r:id="rId10" tooltip="Download interview audio recording for User 1 Selected Candidate"/>
+    <hyperlink ref="K9" r:id="rId9" tooltip="Download interview transcript docx for Aarav Sharma"/>
+    <hyperlink ref="L9" r:id="rId10" tooltip="Download interview audio recording for Aarav Sharma"/>
     <hyperlink ref="K10" r:id="rId11" tooltip="Download interview transcript docx for Snehal Harde"/>
     <hyperlink ref="L10" r:id="rId12" tooltip="Download interview audio recording for Snehal Harde"/>
     <hyperlink ref="K11" r:id="rId13" tooltip="Download interview transcript docx for Snehal Harde"/>

</xml_diff>

<commit_message>
feat: add comprehensive dashboard layout, backend routing, database services, and candidate interview modules
</commit_message>
<xml_diff>
--- a/server/data/reports/Selected_Candidates_2026-10-12.xlsx
+++ b/server/data/reports/Selected_Candidates_2026-10-12.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="56">
   <si>
     <t>AvaHire AI - Daily Selected Candidates Report (12-Oct-2026)</t>
   </si>
   <si>
-    <t>Selection Date: 12-Oct-2026  |  Total Selected: 12 Selected Candidates  |  Generated: 12/10/2026, 19:46:51</t>
+    <t>Selection Date: 12-Oct-2026  |  Total Selected: 12 Selected Candidates  |  Generated: 13/10/2026, 01:49:03</t>
   </si>
   <si>
     <t>Sr. No.</t>
@@ -58,7 +58,7 @@
     <t>Foreign Candidate</t>
   </si>
   <si>
-    <t>foreign.1791794413159@example.com</t>
+    <t>foreign.1791794342458@example.com</t>
   </si>
   <si>
     <t>N/A</t>
@@ -70,7 +70,7 @@
     <t>Product</t>
   </si>
   <si>
-    <t>12 Oct 2026, 14:10</t>
+    <t>12 Oct 2026, 14:09</t>
   </si>
   <si>
     <t>12-Oct-2026</t>
@@ -88,25 +88,28 @@
     <t>Download Recording (Audio)</t>
   </si>
   <si>
-    <t>foreign.1791794342458@example.com</t>
-  </si>
-  <si>
-    <t>12 Oct 2026, 14:09</t>
-  </si>
-  <si>
-    <t>Aarav Sharma</t>
-  </si>
-  <si>
-    <t>aarav.sharma@example.com</t>
-  </si>
-  <si>
-    <t>+91 99887 76655</t>
-  </si>
-  <si>
-    <t>AI Research Scientist</t>
-  </si>
-  <si>
-    <t>AI/ML</t>
+    <t>Divya Nambiar</t>
+  </si>
+  <si>
+    <t>divya.nambiar.1791794342458@example.com</t>
+  </si>
+  <si>
+    <t>Cloud Security Specialist</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Aakash Patel</t>
+  </si>
+  <si>
+    <t>aakash.patel.1791794342458@example.com</t>
+  </si>
+  <si>
+    <t>Senior Frontend Engineer</t>
+  </si>
+  <si>
+    <t>Engineering</t>
   </si>
   <si>
     <t>User 2 Selected Candidate</t>
@@ -124,6 +127,15 @@
     <t>12 Oct 2026, 13:18</t>
   </si>
   <si>
+    <t>User 1 Selected Candidate</t>
+  </si>
+  <si>
+    <t>u1.sel.1791791288048@test.com</t>
+  </si>
+  <si>
+    <t>Full Stack Engineer</t>
+  </si>
+  <si>
     <t>Snehal Harde</t>
   </si>
   <si>
@@ -134,9 +146,6 @@
   </si>
   <si>
     <t>devops</t>
-  </si>
-  <si>
-    <t>Engineering</t>
   </si>
   <si>
     <t>10 Oct 2026, 11:11</t>
@@ -811,22 +820,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>20</v>
@@ -849,22 +858,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>20</v>
@@ -887,22 +896,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>20</v>
@@ -925,22 +934,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>20</v>
@@ -963,22 +972,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>20</v>
@@ -1001,22 +1010,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>20</v>
@@ -1039,22 +1048,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>20</v>
@@ -1077,22 +1086,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>20</v>
@@ -1115,22 +1124,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>20</v>
@@ -1153,7 +1162,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>16</v>
@@ -1162,13 +1171,13 @@
         <v>16</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>20</v>
@@ -1191,22 +1200,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>20</v>
@@ -1232,14 +1241,14 @@
   <hyperlinks>
     <hyperlink ref="K5" r:id="rId1" tooltip="Download interview transcript docx for Foreign Candidate"/>
     <hyperlink ref="L5" r:id="rId2" tooltip="Download interview audio recording for Foreign Candidate"/>
-    <hyperlink ref="K6" r:id="rId3" tooltip="Download interview transcript docx for Foreign Candidate"/>
-    <hyperlink ref="L6" r:id="rId4" tooltip="Download interview audio recording for Foreign Candidate"/>
-    <hyperlink ref="K7" r:id="rId5" tooltip="Download interview transcript docx for Aarav Sharma"/>
-    <hyperlink ref="L7" r:id="rId6" tooltip="Download interview audio recording for Aarav Sharma"/>
+    <hyperlink ref="K6" r:id="rId3" tooltip="Download interview transcript docx for Divya Nambiar"/>
+    <hyperlink ref="L6" r:id="rId4" tooltip="Download interview audio recording for Divya Nambiar"/>
+    <hyperlink ref="K7" r:id="rId5" tooltip="Download interview transcript docx for Aakash Patel"/>
+    <hyperlink ref="L7" r:id="rId6" tooltip="Download interview audio recording for Aakash Patel"/>
     <hyperlink ref="K8" r:id="rId7" tooltip="Download interview transcript docx for User 2 Selected Candidate"/>
     <hyperlink ref="L8" r:id="rId8" tooltip="Download interview audio recording for User 2 Selected Candidate"/>
-    <hyperlink ref="K9" r:id="rId9" tooltip="Download interview transcript docx for Aarav Sharma"/>
-    <hyperlink ref="L9" r:id="rId10" tooltip="Download interview audio recording for Aarav Sharma"/>
+    <hyperlink ref="K9" r:id="rId9" tooltip="Download interview transcript docx for User 1 Selected Candidate"/>
+    <hyperlink ref="L9" r:id="rId10" tooltip="Download interview audio recording for User 1 Selected Candidate"/>
     <hyperlink ref="K10" r:id="rId11" tooltip="Download interview transcript docx for Snehal Harde"/>
     <hyperlink ref="L10" r:id="rId12" tooltip="Download interview audio recording for Snehal Harde"/>
     <hyperlink ref="K11" r:id="rId13" tooltip="Download interview transcript docx for Snehal Harde"/>

</xml_diff>